<commit_message>
ver 4 better desciptions matrix and lil bit new dashboard
</commit_message>
<xml_diff>
--- a/IT_Routing_Matrix_sorted.xlsx
+++ b/IT_Routing_Matrix_sorted.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\muham\OneDrive\Documents\New folder\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\muham\OneDrive\Documents\ai_dispach_excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29056A39-D58C-4059-A5F1-AAE27980072F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24A0E3AF-667F-4106-8714-120AF165276B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,13 +16,14 @@
     <sheet name="Skill_Dictionary" sheetId="1" r:id="rId1"/>
     <sheet name="Staff_Roster" sheetId="2" r:id="rId2"/>
     <sheet name="Queue_Map" sheetId="3" r:id="rId3"/>
+    <sheet name="Ticket_Types" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="398" uniqueCount="150">
   <si>
     <t>Unique_Skill</t>
   </si>
@@ -36,57 +37,30 @@
     <t>Accommodation</t>
   </si>
   <si>
-    <t>IT portals and services related to campus housing and dormitory management</t>
-  </si>
-  <si>
     <t>Admission</t>
   </si>
   <si>
-    <t>Portals and systems handling prospective student applications and enrollment</t>
-  </si>
-  <si>
     <t>All room bookings</t>
   </si>
   <si>
-    <t>IT systems and portals for reserving classrooms, meeting rooms, and lecture halls</t>
-  </si>
-  <si>
     <t>Antivirus_Desktop_Support</t>
   </si>
   <si>
-    <t>Endpoint security, malware removal, and institutional antivirus software management</t>
-  </si>
-  <si>
     <t>Assign storage_Google_Storage</t>
   </si>
   <si>
-    <t>Managing quotas and access for institutional cloud storage (Google Drive, OneDrive) and local servers</t>
-  </si>
-  <si>
     <t>Budget</t>
   </si>
   <si>
-    <t>IT systems for university departmental financial planning and budget allocation</t>
-  </si>
-  <si>
     <t>Bursary</t>
   </si>
   <si>
-    <t>IT systems managing student billing, tuition payments, and financial aid</t>
-  </si>
-  <si>
     <t>COI</t>
   </si>
   <si>
-    <t>University-specific IT application, system, or administrative process</t>
-  </si>
-  <si>
     <t>Campus network (LAN)</t>
   </si>
   <si>
-    <t>Troubleshooting physical local network connections, switches, and ethernet drops</t>
-  </si>
-  <si>
     <t>Charging_Application</t>
   </si>
   <si>
@@ -114,126 +88,60 @@
     <t>ERP</t>
   </si>
   <si>
-    <t>Enterprise Resource Planning systems (backend systems for HR, finance, and university operations)</t>
-  </si>
-  <si>
-    <t>ERP setup_Desktop_Support</t>
-  </si>
-  <si>
-    <t>Installation, configuration, and user access management for ERP client software</t>
-  </si>
-  <si>
     <t>Email</t>
   </si>
   <si>
-    <t>Management of university email accounts, routing issues, spam filtering, and client configuration</t>
-  </si>
-  <si>
     <t>Finance form (DMS)</t>
   </si>
   <si>
     <t>General_Application</t>
   </si>
   <si>
-    <t>Standard Application support, general inquiries, and cross-functional ticket escalation</t>
-  </si>
-  <si>
     <t>General_Desktop_Support</t>
   </si>
   <si>
-    <t>Standard Desktop Support support, general inquiries, and cross-functional ticket escalation</t>
-  </si>
-  <si>
     <t>General_Email_Mailing_List</t>
   </si>
   <si>
-    <t>Standard Email/Mailing List support, general inquiries, and cross-functional ticket escalation</t>
-  </si>
-  <si>
     <t>General_FTTH</t>
   </si>
   <si>
-    <t>Standard FTTH support, general inquiries, and cross-functional ticket escalation</t>
-  </si>
-  <si>
     <t>General_Google_Storage</t>
   </si>
   <si>
-    <t>Standard Google Storage support, general inquiries, and cross-functional ticket escalation</t>
-  </si>
-  <si>
     <t>General_IPPhone</t>
   </si>
   <si>
-    <t>Standard IPPhone support, general inquiries, and cross-functional ticket escalation</t>
-  </si>
-  <si>
     <t>General_Infra</t>
   </si>
   <si>
-    <t>Standard Infra support, general inquiries, and cross-functional ticket escalation</t>
-  </si>
-  <si>
     <t>General_IoT</t>
   </si>
   <si>
-    <t>Standard IoT support, general inquiries, and cross-functional ticket escalation</t>
-  </si>
-  <si>
     <t>General_Plagiarism_Check</t>
   </si>
   <si>
-    <t>Standard Plagiarism Check support, general inquiries, and cross-functional ticket escalation</t>
-  </si>
-  <si>
     <t>General_User_account</t>
   </si>
   <si>
-    <t>Standard User account support, general inquiries, and cross-functional ticket escalation</t>
-  </si>
-  <si>
     <t>General_VM_Request</t>
   </si>
   <si>
-    <t>Standard VM Request support, general inquiries, and cross-functional ticket escalation</t>
-  </si>
-  <si>
     <t>General_Web_Hosting</t>
   </si>
   <si>
-    <t>Standard Web Hosting support, general inquiries, and cross-functional ticket escalation</t>
-  </si>
-  <si>
     <t>IPPhone</t>
   </si>
   <si>
-    <t>Voice over IP (VoIP) telephony services for faculty and staff offices</t>
-  </si>
-  <si>
-    <t>Internet connection</t>
-  </si>
-  <si>
-    <t>Managing external ISP links, bandwidth, and general campus-wide internet availability</t>
-  </si>
-  <si>
     <t>Internet servers</t>
   </si>
   <si>
-    <t>Maintenance of outward-facing and internal university servers (web hosting, DNS, virtual hosting)</t>
-  </si>
-  <si>
     <t>Internet service in residential areas</t>
   </si>
   <si>
-    <t>Troubleshooting wired and wireless (Wi-Fi) internet connectivity in student dorms</t>
-  </si>
-  <si>
     <t>PC support including Windows_Desktop_Support</t>
   </si>
   <si>
-    <t>Hardware troubleshooting, OS installation, and desktop/laptop support for staff and labs</t>
-  </si>
-  <si>
     <t>PE</t>
   </si>
   <si>
@@ -243,27 +151,15 @@
     <t>Payroll</t>
   </si>
   <si>
-    <t>IT systems managing staff/faculty salaries, timesheets, and compensation</t>
-  </si>
-  <si>
     <t>Phone billing system</t>
   </si>
   <si>
-    <t>Tracking and invoicing for institutional telecommunications and phone usage</t>
-  </si>
-  <si>
-    <t>Plagiarism check</t>
-  </si>
-  <si>
     <t>SAS</t>
   </si>
   <si>
     <t>SCPO</t>
   </si>
   <si>
-    <t>Sponsored and Contracted Projects Office IT systems and administration</t>
-  </si>
-  <si>
     <t>SIS</t>
   </si>
   <si>
@@ -273,24 +169,15 @@
     <t>Software licenses_Desktop_Support</t>
   </si>
   <si>
-    <t>Turnitin software</t>
-  </si>
-  <si>
     <t>User account</t>
   </si>
   <si>
-    <t>Password resets, new account creation, and SSO / Active Directory management</t>
-  </si>
-  <si>
     <t>VM setup_VM_Request</t>
   </si>
   <si>
     <t>VM setup_Web_Hosting</t>
   </si>
   <si>
-    <t>Provisioning and architecture setup of virtual machines for web hosting.</t>
-  </si>
-  <si>
     <t>WP setup</t>
   </si>
   <si>
@@ -300,15 +187,6 @@
     <t>hardware/network</t>
   </si>
   <si>
-    <t>Hardware troubleshooting and IoT network connectivity.</t>
-  </si>
-  <si>
-    <t>mailing list</t>
-  </si>
-  <si>
-    <t>software license_Desktop_Support</t>
-  </si>
-  <si>
     <t>Owner</t>
   </si>
   <si>
@@ -381,79 +259,220 @@
     <t>Web Hosting</t>
   </si>
   <si>
-    <t>Technical support for academic integrity and anti-plagiarism software</t>
-  </si>
-  <si>
-    <t>Turnitin application, system, or administrative process</t>
-  </si>
-  <si>
-    <t>A system to record the conflict of interests of every employee.</t>
-  </si>
-  <si>
-    <t>Central, software-based engine for Cisco's IP phones</t>
-  </si>
-  <si>
-    <t>Performance Evaluation System is the system for evaluating the performance of staff.</t>
-  </si>
-  <si>
-    <t>Partnership Management Information System is still not opened yet but will be used to keep all agreements AIT has with different organizations and companies around the world.</t>
-  </si>
-  <si>
-    <t>Student Assistantship System is a system for hiring student assistants. Therefore student contracts and timesheets are the main components.</t>
-  </si>
-  <si>
-    <t>System for recording student records such as admissions, course enrollments, grades, transcripts, student clearance, student invoices, course evaluation. For every student except School of Management students.</t>
-  </si>
-  <si>
-    <t>System for recording student records such as admissions, course enrollments, grades, transcripts, student clearance, student invoices, course evaluation. For only School of Management students.</t>
-  </si>
-  <si>
-    <t>Provisioning and configuring Virtual Machines.</t>
-  </si>
-  <si>
-    <t>Provisioning, auditing, and distributing paid software and.</t>
-  </si>
-  <si>
-    <t>Creation and management of departmental or course-specific email distribution groups.</t>
-  </si>
-  <si>
-    <t>Administration of the broader university network infrastructure, routing, and firewalls.</t>
-  </si>
-  <si>
-    <t>WordPress installation, configuration etc.</t>
-  </si>
-  <si>
-    <t>AIT International School. AITIS is an application we developed for admission and invoicing systems.</t>
-  </si>
-  <si>
-    <t>Billing, invoicing, and cross-charging departments for things related to applications.</t>
-  </si>
-  <si>
-    <t>Billing, invoicing, and cross-charging departments for things related to Virtual machine requests.</t>
-  </si>
-  <si>
-    <t>Billing, invoicing, and cross-charging departments for things related to desktop support.</t>
-  </si>
-  <si>
-    <t>Billing, invoicing, and cross-charging departments for things related to FTTH.</t>
-  </si>
-  <si>
-    <t>Billing, invoicing, and cross-charging departments for things related to Google storage.</t>
-  </si>
-  <si>
-    <t>Billing, invoicing, and cross-charging departments for things related to IPPhone.</t>
-  </si>
-  <si>
-    <t>Billing, invoicing, and cross-charging departments for things related to Infrastructure.</t>
-  </si>
-  <si>
     <t>Campus network (Wifi)</t>
   </si>
   <si>
-    <t>Provisioning, auditing, and distributing paid software.</t>
-  </si>
-  <si>
-    <t>Troubleshooting  campus Wi-Fi access points</t>
+    <t>[TYPE: Task] [SCOPE: Billing Only] Financial invoicing, accounting entries, and cross-charging departments for software and applications.</t>
+  </si>
+  <si>
+    <t>[TYPE: Task] [SCOPE: Billing Only] Financial invoicing, accounting entries, and cross-charging departments for hardware and desktop services.</t>
+  </si>
+  <si>
+    <t>[TYPE: Task] [SCOPE: Billing Only] Financial invoicing, accounting entries, and cross-charging departments for extended cloud storage quotas.</t>
+  </si>
+  <si>
+    <t>[TYPE: Task] [SCOPE: Billing Only] Financial invoicing, accounting entries, and cross-charging departments for physical phone lines and hardware provisioning.</t>
+  </si>
+  <si>
+    <t>[TYPE: Task] [SCOPE: Billing Only] Financial invoicing, accounting entries, and cross-charging departments for core server hosting and network architecture projects.</t>
+  </si>
+  <si>
+    <t>[TYPE: Task] [SCOPE: Billing Only] Financial invoicing, accounting entries, and cross-charging departments for virtual machine environments.</t>
+  </si>
+  <si>
+    <t>[TYPE: Task] [LEVEL: Senior Escalation Only - Harianto] Enterprise hardware audits, mass software distribution failures, and vendor escalated support. DO NOT use for individual PC slow symptoms.</t>
+  </si>
+  <si>
+    <t>[TYPE: System] [LEVEL: Senior Escalation Only - Harianto] Master email relay server architecture failures, institutional spam filtering breaches, or backend security locks.</t>
+  </si>
+  <si>
+    <t>[TYPE: Task] [LEVEL: Senior Escalation Only - Viraphan] Core fiber distribution hub breakdowns, main optical line breaks, or broad residential grid failures.</t>
+  </si>
+  <si>
+    <t>[TYPE: System] [LEVEL: Senior Escalation Only - Harianto] Global tenant admin console configuration, tenant wide quota policy adjustments, or compliance audits.</t>
+  </si>
+  <si>
+    <t>[TYPE: System] [LEVEL: Senior Escalation Only - Harianto / Viraphan] Central telephone exchange hardware downtime, trunk line drops, or severe platform communication crashes.</t>
+  </si>
+  <si>
+    <t>[TYPE: System] [LEVEL: Senior Escalation Only - Viraphan] Main campus backbone network outages, primary routing switch updates, core firewalls, or master datacenter power failures.</t>
+  </si>
+  <si>
+    <t>[TYPE: System] [LEVEL: Senior Escalation Only - Viraphan] Core smart campus IoT platform structural outages, controller failures, or central sensor array drops.</t>
+  </si>
+  <si>
+    <t>[TYPE: System] [LEVEL: Senior Escalation Only - Harianto] Global Turnitin contract compliance auditing, system-wide licensing freezes, or enterprise API failures.</t>
+  </si>
+  <si>
+    <t>[TYPE: System] [LEVEL: Senior Escalation Only - Harianto] Active Directory schema modifications, master domain controller dropouts, or cross-realm authentication failures.</t>
+  </si>
+  <si>
+    <t>[TYPE: System] [LEVEL: Senior Escalation Only - Viraphan] Structural host capacity planning, enterprise hypervisor cluster provisioning, or master datacenter resource rebalancing.</t>
+  </si>
+  <si>
+    <t>[TYPE: System] [LEVEL: Senior Escalation Only - Harianto] Main campus web server cluster outages, reverse proxy failures, or tenant-wide control panel service drops.</t>
+  </si>
+  <si>
+    <t>[TYPE: System] [AUTH: Global Master Account] AIT International School (AITIS) system management. INCLUDES: AITIS system administration, student invoicing workflows within AITIS, international school student admissions tracking, and AITIS platform-specific errors. EXCLUDES: General school tasks, master AIT account lockouts, and all standard login/password problems (route to User account queue). KEYWORDS: AITIS, international school, student invoicing, AIT International School, admissions.</t>
+  </si>
+  <si>
+    <t>[TYPE: System] [AUTH: Global Master Account] Core portals handling prospective student applications, tracking, and university enrollment pipelines. INCLUDES: Technical support for admission.ait.ac.th, applicant portal errors, digital application tracking workflows, and online enrollment pipeline system configurations. EXCLUDES: AIT International School (AITIS) admissions, general academic registration systems, and master AIT account lockouts. KEYWORDS: admission.ait.ac.th, admission, prospective student, application pipeline, enrollment portal.</t>
+  </si>
+  <si>
+    <t>[TYPE: System] [AUTH: Global Master Account] Accommodation Portal and Housing Management System. INCLUDES: Technical support and online services for ofam.ait.ac.th, campus housing portals, dormitory room management website issues, digital accommodation application errors, and ofam system administration. EXCLUDES: Physical housing maintenance (e.g., broken locks, plumbing, AC repairs), physical Wi-Fi drops or dormitory internet connectivity issues, and master AIT account lockouts. KEYWORDS: ofam.ait.ac.th, ofam, accommodation, campus housing, dormitory room management, housing portal.</t>
+  </si>
+  <si>
+    <t>[TYPE: System] [AUTH: Global Master Account] IT systems and central portals for reserving classrooms, meeting spaces, and lecture halls. INCLUDES: All digital room booking system configurations, online reservation portals, technical issues with apps.ait.ac.th/roombooking, classroom/meeting space reservation software errors, and digital scheduling workflows. EXCLUDES: Physical room maintenance, AV/projector hardware troubleshooting inside the rooms, physical key management, and master AIT account lockouts. KEYWORDS: room booking, roombooking, apps.ait.ac.th/roombooking, reserve classroom, meeting space reservation, booking system.</t>
+  </si>
+  <si>
+    <t>[TYPE: System] [AUTH: Global Master Account] IT software platforms used for university department financial planning and corporate budget allocation. INCLUDES: Technical administration of the university-wide budget system, troubleshooting portal interface errors, online software access issues for financial planning modules, and digital allocation system workflow configurations. EXCLUDES: Inquiries regarding actual physical money, offline accounting paperwork, physical procurement approvals, and master AIT account lockouts. KEYWORDS: budget system, financial planning software, budget allocation portal, corporate budget module.</t>
+  </si>
+  <si>
+    <t>[TYPE: System] [AUTH: Global Master Account] IT financial frameworks managing student billing, tuition payment portals, and financial aid tracking. INCLUDES: Technical administration of the online bursary portal, student billing interface errors, digital tuition payment gateway issues, financial aid tracking software configurations, and system-side invoicing workflows. EXCLUDES: Physical cash handling, offline refund processing, specific fee policy disputes, and master AIT account lockouts. KEYWORDS: bursary portal, tuition payment system, student billing software, financial aid portal, invoicing system.</t>
+  </si>
+  <si>
+    <t>[TYPE: System] [AUTH: Global Master Account] Conflict of Interest application portal. Used exclusively by university employees to record and submit organization disclosures. INCLUDES: Technical support for the digital COI submission portal, online form errors, tracking system workflow bottlenecks, website interface bugs, and employee access permissions within the disclosure tool. EXCLUDES: Reviewing the actual content of disclosures, legal policy compliance advice, human resource investigations, and master AIT account lockouts. KEYWORDS: COI, conflict of interest, disclosure portal, submission system, organization disclosure tool.</t>
+  </si>
+  <si>
+    <t>[TYPE: Task] Endpoint antivirus installation, local malware scanning, virus removal, and user-initiated device security support. INCLUDES: Individual user requests for virus removal, troubleshooting antivirus software installations, manual malware scans on infected user laptops/desktops, local security alert remediation, and remote assistance for virus fixing. EXCLUDES: Campus-wide cyber attacks, server-level firewall breaches, network penetration testing, institutional security policy changes, and master AIT account lockouts. KEYWORDS: virus, antivirus, malware, virus removal, infection, scan, remote fix, infected device, malware bytes, defender.</t>
+  </si>
+  <si>
+    <t>[TYPE: System] Core maintenance, patching, and OS setup of outward-facing and internal university servers (DNS, central web server farms, load balancers). INCLUDES: High-level administration of DNS zone files, global load balancer configurations, core university web server farm crashes, critical server operating system patching, and central data center virtual machine provisioning. EXCLUDES: Individual website content updates, local desktop database application setup, network switch port wiring, and master AIT account lockouts. KEYWORDS: DNS server, web server farm, load balancer, server patching, core server maintenance, zone configuration, data center VM.</t>
+  </si>
+  <si>
+    <t>[TYPE: Task] Desktop and laptop hardware component failures, operating system crashes, blue screens, slow computer symptoms, and office peripheral wiring across all workstations. INCLUDES: All kinds of desktop support, troubleshooting, local configurations, and remote configuration for desktops, staff laptops, and lab computers. EXCLUDES: Server infrastructure maintenance, campus-wide network upgrades, personal non-university student devices, ERP/HSMART account management, and master AIT account lockouts. KEYWORDS: PC support, Windows crash, blue screen, BSOD, slow computer, hardware failure, university computer, office laptop, desktop freezing, workstation repair, remote support, desktop config.</t>
+  </si>
+  <si>
+    <t>[TYPE: System] [AUTH: Global Master Account] Performance Evaluation software framework used by human resources to monitor and evaluate employee benchmarks. INCLUDES: Technical administration of the digital PE appraisal portal, system form submission errors, evaluation workflow step routing bugs, and module configuration issues inside the evaluation tracking system. EXCLUDES: Physical performance review discussions, manual HR filing, salary renegotiations, and master AIT account lockouts. KEYWORDS: PE system, performance evaluation portal, appraisal software, employee benchmarks, evaluation workflow.</t>
+  </si>
+  <si>
+    <t>[TYPE: System] [AUTH: Global Master Account] Partnership Management Information System used for tracking organizational contracts, international agreements, and corporate partnerships globally. INCLUDES: System administration of the PMIS tracking database, online contract record save errors, digital MoU upload workflows, profile permission settings within the partnership portal, and global data interface bugs. EXCLUDES: External legal advice, negotiating contract terms face-to-face, manual partnership signing ceremonies, and master AIT account lockouts. KEYWORDS: PMIS, partnership management system, contract tracking portal, international agreement software, corporate partnership tool.</t>
+  </si>
+  <si>
+    <t>[TYPE: System] [AUTH: Global Master Account] IT payroll application portal managing employee monthly compensation tracking, historical salary slips, and payroll sheets. INCLUDES: Technical platform administration, online payslip rendering bugs, electronic salary sheet processing failures, automated deduction profile settings, and portal interface errors. EXCLUDES: Physical cash distribution, manual salary bank transfers, direct tax policy disputes, and master AIT account lockouts. KEYWORDS: payroll system, payslip portal, salary tracking software, compensation application, digital payslip error.</t>
+  </si>
+  <si>
+    <t>[TYPE: Task] Tracking, logging, and processing department charges for external calls made from campus IP phones. INCLUDES: Monitoring external phone call logs, resolving billing discrepancy tickets for outgoing long-distance or external calls, assigning call-related expenses to departmental cost centers, and troubleshooting internal invoicing errors for phone expenditures. EXCLUDES: Physical IP phone hardware repairs, setting up new phone extensions, central Cisco telephony server provisioning, and master AIT account lockouts. KEYWORDS: phone billing, call logs, external call charges, phone expenditure, long distance bill, phone invoice, call tracking.</t>
+  </si>
+  <si>
+    <t>[TYPE: System] [AUTH: Global Master Account] Student Assistantship System platform handling student employment agreements, hourly job contracts, and student timesheet submittals. INCLUDES: Technical administration of the digital SAS platform, timesheet data submission errors, digital employment contract generation failure bugs, and portal approval workflow routing issues. EXCLUDES: Physical student hiring interviews, actual hourly wage calculation approvals, human resource policy disputes, and master AIT account lockouts. KEYWORDS: SAS system, student assistantship portal, student timesheet software, job contract workflow, student employment application.</t>
+  </si>
+  <si>
+    <t>[TYPE: System] [AUTH: Global Master Account] Sponsored and Contracted Projects Office management app used for monitoring research grants, fiscal compliance, and project tracking. INCLUDES: Application support for the SCPO portal, digital grant tracking database errors, fiscal compliance entry submission failures, and milestone verification workflow bugs. EXCLUDES: Reviewing actual scientific research content, physical grant budget allocation decisions, writing research proposals, and master AIT account lockouts. KEYWORDS: SCPO, research grant portal, project tracking application, fiscal compliance software, project monitoring tool.</t>
+  </si>
+  <si>
+    <t>[TYPE: System] [AUTH: Global Master Account] Student Information System application portal handling course enrollments, grade viewing, official transcripts, and clearance workflows. INCLUDES: Central platform support  course registration portal errors, transcript rendering bugs, digital clearance workflow failures, and interface issues inside the core SIS module. EXCLUDES: Specific School of Management system portals (SOMSIS), course curriculum updates, face-to-face academic advising, and master AIT account lockouts. KEYWORDS: SIS, Student Information System, course enrollment, view grades, official transcripts, student clearance workflow.</t>
+  </si>
+  <si>
+    <t>[TYPE: System] [AUTH: Global Master Account] School of Management Student Information System application portal handling admissions, enrollment, grade viewing, transcripts, and financial invoice. INCLUDES: Technical system-level support tailored explicitly for the School of Management's portal modules, management student registration errors, SOM transcript extraction issues, and portal-side invoice generation crashes. EXCLUDES: General university student data systems (SIS), processing actual cash or card payments, physical student counseling, and master AIT account lockouts. KEYWORDS: SOMSIS, School of Management portal, SOM enrollment, management student system, SOM grades, management school invoice.</t>
+  </si>
+  <si>
+    <t>[TYPE: Task] Allocating specific resources, provisioning virtual operating environments, and configuring new Virtual Machine instances for projects. INCLUDES: All kinds of general virtual machine creation, processing VM resource allocation requests (CPU, RAM, storage) for academic or departmental projects, initializing baseline operating system environments (Linux/Windows server instances), granting remote desktop or SSH access to the requesting user, and modifying general VM session parameters. EXCLUDES: Configuring public-facing web domain names, deploying specialized web-hosting software stacks, central datacenter hypervisor-level master maintenance, and master AIT account lockouts. KEYWORDS: VM request, create virtual machine, allocate resources, project VM, provision instance, OS environment, session access, virtual server setup.</t>
+  </si>
+  <si>
+    <t>[TYPE: System] [AUTH: Global Master Account] Management of corporate university email accounts, client connectivity profile setup, and security filters. INCLUDES: Centralized administration of the mail server infrastructure, mailing list creation and configuration, global spam/security filters, mail routing errors, and domain-level email delivery issues. EXCLUDES: Individual user desktop email application setups (e.g., configuring Outlook or Thunderbird on a local PC) and user account password resets. KEYWORDS: email system, mailing list, webmail, mail server, spam filter, mx records, email domain, create group email.</t>
+  </si>
+  <si>
+    <t>[TYPE: Task] Specific virtual machine environment architecture setup and configuration optimized for web hosting deployment. INCLUDES: All kinds of VM environment provisioning and architectural preparation for hosting websites, configuring virtual hardware parameters or network layers to support heavy web traffic, setting up specific server security groups/ports for web protocols (HTTP/HTTPS), binding base IP addresses, and preparing the virtual directory mapping so the instance is ready for a web hosting stack or CMS installation. EXCLUDES: Actually installing or configuring web applications or content management software (like WordPress, Apache, Nginx, or IIS), managing active live databases, deploying actual website code, setting up SSL certificates, and master AIT account lockouts. KEYWORDS: web hosting VM setup, prepare web VM, web traffic configuration, port configuration, virtual machine for hosting, web server preparation, hosting environment setup.</t>
+  </si>
+  <si>
+    <t>[TYPE: Task] WordPress content management system local installation, configuration wizard setup, database bindings, and theme activations. INCLUDES: All kinds of WordPress setups and platform-level configurations, downloading and unpacking core WP installation files onto the web server, running the initial web configuration setup wizard, linking the application to its local or remote MySQL/MariaDB database, activating default or custom institutional themes, and setting up initial administrative dashboard logins. EXCLUDES: Server infrastructure-level virtualization provisioning, OS-level firewall adjustments, raw domain name registrations, physical web cluster adjustments, and master network account lockouts. KEYWORDS: WP setup, install WordPress, WordPress configuration, database binding, theme activation, CMS installation, WordPress wizard, setup WP site.</t>
+  </si>
+  <si>
+    <t>[TYPE: Task] Physical hardware troubleshooting, peripheral replacements, and network connectivity configurations for specialized IoT equipment. INCLUDES: All kinds of hardware and network configuration work requiring an IoT specialist, setting up internet-of-things devices, configuring network pathways for specialized smart equipment (such as biometric scanners, environmental sensors, IP cameras, or smart office displays), and troubleshooting hardware integrations for network-connected campus systems. EXCLUDES: Deep-layer core network engineering, global enterprise firewall architecture modifications, campus-wide internet routing maintenance, and master AIT account lockouts. KEYWORDS: IoT specialist, hardware network, IoT setup, smart device configuration, sensor network, biometric integration, network hardware, specialized IoT support.</t>
+  </si>
+  <si>
+    <t>[TYPE: System] Central server software management and virtual provisioning of Cisco IP Phone profiles. INCLUDES: Device registration on the central telephony server, softphone virtual configuration profiles, managing remote extension assignments on the network, firmware deployment pushes, and server-side telephony system errors. EXCLUDES: Physical desk phone hardware troubleshooting, on-site device installations, broken handset replacements, static on physical lines,telephone installation, and master AIT account lockouts. KEYWORDS: IPPhone system, virtual provisioning, phone profile, registration error, telephony server.</t>
+  </si>
+  <si>
+    <t>[TYPE: Core Infrastructure] [LEVEL: Admin/High-Level] Global campus internet bandwidth, ISP (Internet Service Provider) links, core firewall routing, and massive campus-wide internet outages. INCLUDES: Core router configurations, BGP/ISP failovers, modifying global firewall traffic rules, and investigating total campus network blackouts. EXCLUDES: Individual user Wi-Fi problems, guest Wi-Fi creation, personal laptop/phone connectivity issues, dropping wireless signal in a specific room, and LAN cable issues. KEYWORDS: ISP, core internet, firewall routing, global outage, campus-wide down, gateway, backbone.</t>
+  </si>
+  <si>
+    <t>[TYPE: System] [AUTH: Finance/Administration] Technical support and access troubleshooting specifically for the AIT Document Management System (DMS) portal and financial approval workflows. INCLUDES: Cannot access apps1.ait.ac.th/dms, errors inside the DMS menu, electronic finance approval forms, and budget/payment tracking sheets. EXCLUDES: General web forms, Google Forms, Microsoft Forms, survey links, admission application forms (route to Admission), and housing request forms (route to Accommodation). DO NOT route here just because the word 'form' is used unless it is explicitly a financial or DMS system form. KEYWORDS: DMS form, apps1.ait.ac.th/dms, finance online form, DMS menu, budget approval form.</t>
+  </si>
+  <si>
+    <t>Problem Solving</t>
+  </si>
+  <si>
+    <t>New Installation</t>
+  </si>
+  <si>
+    <t>Provide Guide/Advise</t>
+  </si>
+  <si>
+    <t>Special Request</t>
+  </si>
+  <si>
+    <t>Ticket_Type</t>
+  </si>
+  <si>
+    <t>A user is asking IT to perform a task. Requests for granting access, modifying accounts, releasing IPs, or providing standard IT services.</t>
+  </si>
+  <si>
+    <t>Something is broken. Troubleshooting technical bugs, service disruptions, error screens, or fixing broken configurations.</t>
+  </si>
+  <si>
+    <t>Setting up brand new hardware, deploying a new workstation, or installing new software from scratch.</t>
+  </si>
+  <si>
+    <t>The user is just asking a question. General how-to questions, seeking instructions, or requesting documentation.</t>
+  </si>
+  <si>
+    <t>[TYPE: Task] Physical wired internet connectivity for office desks and specific rooms. INCLUDES: Dead LAN ports in the wall, broken ethernet cables, requesting a new LAN port activation, wired internet dropping on a single office PC. EXCLUDES: Wireless/Wi-Fi issues, eduroam, core ISP outages, and global firewall routing. KEYWORDS: LAN port, ethernet cable, wall jack, wired internet, network cable, activate port.</t>
+  </si>
+  <si>
+    <t>[TYPE: Task] [AUTH: Global Master Account] The master identity boundary managing all user accounts, profile data, credentials, and digital identities for students, professors, and staff across all university systems. INCLUDES: All kinds of user account-related work, troubleshooting profile data sync bugs, managing user identity records mapped to university campus cards, resetting forgotten passwords, resolving multi-factor authentication (MFA) locks, unlocking single sign-on (SSO) or Active Directory accounts, and fixing login blockages on all university platforms. EXCLUDES: ERP/HSMART application login failures, local ERP account registration, ERP access, physical card replacement printing, computer hardware setups, and master network server maintenance. KEYWORDS: user account, identity data, student account, staff account, professor login, campus card data, password reset, unlock account, MFA lock, SSO access, Active Directory profile, credential issue.</t>
+  </si>
+  <si>
+    <t>[TYPE: Task] Manages the campus IP telephony ecosystem end-to-end, including physical desk phone hardware, telephone line configurations, and extension/directory number changes. INCLUDES: Installing physical desk phones, configuring hardware handsets, setting up telephone extensions, updating staff phone directory lines, fixing dead desktop phone screens, troubleshooting static or no dial tone on office phones, and handling general hardware/line failures. EXCLUDES: Softphone software troubleshooting (e.g., Cisco Webex or Jabber app errors on laptops), mobile phone cellular network issues, and master AIT account lockouts. KEYWORDS: Cisco phone, IPPhone, desk phone, extension,call forwarding, extension, telephone set, new telephone installation</t>
+  </si>
+  <si>
+    <t>[TYPE: Task] Oversee validation, legal key registration, corporate license allocation, and deployment of institutional software suites (including Microsoft Office, ERP systems, Canva, and Google Workspace, Zoom). INCLUDES: Directing users on how to download institutional applications, providing step-by-step instructions for license activation, assigning available product keys to staff devices, and troubleshooting validation errors or expired software license warnings. EXCLUDES: Reviewing legal corporate contract terms with vendors, purchasing non-standard retail software licenses, server-level enterprise license server configurations, and master AIT account lockouts. KEYWORDS: software license, product key, activate Office, license validation, download software, software activation error, Canva license, software instruction, Zoom Pro.</t>
+  </si>
+  <si>
+    <t>[TYPE: Task] Installation, configuration, client software loading, and endpoint troubleshooting for ERP local client installations. INCLUDES: All kinds of desktop support, troubleshooting, local installations, and remote configuration to set up ERP client software on university-owned office devices or staff laptops; resolving database connection settings on user devices; and fixing local application loading errors. EXCLUDES: ERP system account creation, HSMART portal password resets, server-side database maintenance,login failures or password issues, and master network account lockouts. KEYWORDS: ERP setup, install ERP, ERP client, local installation, remote desktop setup, configure ERP software, HSMART client, desktop config.</t>
+  </si>
+  <si>
+    <t>[TYPE: Task] Wireless network access and troubleshooting for academic buildings, devices, or specific rooms/events. INCLUDES: AIT Wi-Fi (AITsec, eduroam), guest Wi-Fi account creation, event/conference Wi-Fi setup, weak wireless signals in specific rooms, and restarting local Access Points (APs). EXCLUDES: Campus-wide internet backbone outages, ISP failures, firewall rule changes,dormitory/student village(SV) Wifi,dormitory/student village(SV) routers and physical LAN port installations. KEYWORDS: Wi-Fi down, guest Wi-Fi, eduroam, wireless signal, AITsec, event Wi-Fi, connect phone to wifi, cannot connect laptop, SSID, Guest Access, Eduroam, Wireless, router.</t>
+  </si>
+  <si>
+    <t>[TYPE: System] [AUTH: Global Master Account] IT backend administration of the Turnitin platform. INCLUDES: Creating instructor profiles, generating Class IDs and Enrollment Keys, fixing login/SSO errors, and resolving software outages. EXCLUDES: Performing actual similarity/plagiarism checks, checking AI scores, generating similarity reports, or evaluating indexes on documents for users.</t>
+  </si>
+  <si>
+    <t>[TYPE: Task] Fulfilling manual requests to scan documents for academic integrity using Turnitin. INCLUDES: Running student or faculty theses/papers through Turnitin, generating similarity reports, checking AI scores, evaluating similarity indexes, and excluding previous work from a similarity check. EXCLUDES: Turnitin account creation, password resets, Class ID setups, or fixing software errors.</t>
+  </si>
+  <si>
+    <t>Plagiarism, AI &amp; Similarity Check (Turnitin)</t>
+  </si>
+  <si>
+    <t>[TYPE: Task] Provisioning, member management, moderation setup, and technical configuration of departmental or course-specific email distribution groups. INCLUDES: All kinds of mailing list-related work, creating new communication groups, adding or removing users from subscription rosters, adjusting list moderation permissions,email group setup, and troubleshooting delivery bounce-backs or distribution sync errors for specific university departments or classes. EXCLUDES: Central email server domain-level infrastructure maintenance, global corporate spam filter adjustments, individual personal mailbox creation, and master network account lockouts. KEYWORDS: mailing list, email group, distribution list, member management, subscriber roster, group communication, list moderation, list sync error.</t>
+  </si>
+  <si>
+    <t>[TYPE: Task] Fulfilling user requests regarding Google cloud storage capacity, shared spaces, and storage allocation adjustments. INCLUDES: Increasing or decreasing individual user storage limits, creating or modifying Google Shared Drives, changing user storage policy tier/plans, and troubleshooting "out of storage" error tickets for Google Workspace accounts. EXCLUDES: OneDrive storage, local hard drive partitions or local enterprise server storage allocation,other Google apps/platform that are not Google storage related, and master AIT account lockouts. KEYWORDS: Google storage, storage plan, quota limit, change storage space, Google Drive, Shared Drives, full storage, increase quota.</t>
+  </si>
+  <si>
+    <t>Core Backbone &amp; ISP Routing</t>
+  </si>
+  <si>
+    <t>[TYPE: Task] Handles internal network troubleshooting across all university residential areas (including Student Dormitories and Faculty Housing/FTTH), resolving localized connectivity issues. INCLUDES: Fixing internet connectivity issues, Wi-Fi drops, and local network ports specifically inside dorm rooms (e.g., L-Dorm, M-Dorm), student housing facilities, student village (e.g., SV01B1) with Wifi related request, and faculty residential zones. EXCLUDES: Network troubleshooting or Wi-Fi connectivity drops in academic buildings (classrooms, lecture halls, administrative offices), campus-wide core network outages, and master AIT account lockouts. KEYWORDS: residential internet, dorm wifi, faculty housing internet, FTTH, room internet, dormitory wifi drop, student village(SV), student housing network, L-Dorm, M-Dorm.</t>
+  </si>
+  <si>
+    <t>ERP Software Installation (Desktop Support)</t>
+  </si>
+  <si>
+    <t>[TYPE: Task] [SCOPE: Billing Only] Financial invoicing, accounting entries, and cross-charging departments for residential fiber-to-the-home connections. INCLUDES: Billing inquiries for dormitories, accommodation move-out charges, fees for damaged Wi-Fi routers in student rooms, and THB invoice disputes. EXCLUDES: Technical troubleshooting of dead internet connections.</t>
+  </si>
+  <si>
+    <t>Mailing Lists &amp; Google Groups Setup</t>
+  </si>
+  <si>
+    <t>Turnitin Backend Administration</t>
+  </si>
+  <si>
+    <t>[TYPE: System] [AUTH: Local ERP Management] Enterprise Resource Planning system managing university institutional resources, finance, and corporate operations. INCLUDES: All technical administration of the ERP platform, ERP-specific user account creation, HSMART user access privileges, module-specific permissions, portal navigation bugs,password resets, forgotten passwords, and all ERP/HSMART login failures or account lockouts. EXCLUDES: General university network account lockouts, external non-ERP software permission requests, and physical accounting or human resource paperwork. KEYWORDS: ERP, HSMART, ERP login, ERP account, module permissions, ERP access, institutional resource system.</t>
+  </si>
+  <si>
+    <t>[TYPE: System] [LEVEL: Senior Escalation Only - Harianto] Critical database failures, app compliance audits, or core multi-system crashes, also serving as the absolute last-resort fallback for unmatched orphan requests. INCLUDES: Database errors, core system crashes, app compliance audits, miscellaneous university web forms, Google Forms, Microsoft Forms, student exit surveys, online surveys,Moodle, Learning Management Systems (LMS), and generic portal configurations not matching any specific system or task skill. EXCLUDES: Routine bugs or access issues for specific known university systems (e.g., SIS, SAS, ERP, Finance form DMS), admission application forms (route to Admission), and housing requests (route to Accommodation). DO NOT route routine application bugs here; specific system skills must be searched first. Use this for forms or surveys ONLY when no other specific system or task queue matches. KEYWORDS: database failure, core crash, compliance audit, exit survey, online survey, generic form,moodle, web form, unmatched portal.</t>
   </si>
 </sst>
 </file>
@@ -793,11 +812,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B60"/>
+  <dimension ref="A1:B58"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="43" customWidth="1"/>
-    <col min="2" max="2" width="99.21875" customWidth="1"/>
+    <col min="1" max="1" width="28.5546875" customWidth="1"/>
+    <col min="2" max="2" width="160.77734375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
@@ -813,7 +832,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>133</v>
+        <v>96</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
@@ -821,463 +840,447 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>4</v>
+        <v>98</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>6</v>
+        <v>97</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>8</v>
+        <v>99</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>10</v>
+        <v>103</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="B7" t="s">
-        <v>12</v>
+        <v>141</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>14</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="B9" t="s">
-        <v>16</v>
+        <v>101</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="B10" t="s">
-        <v>121</v>
+        <v>102</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>141</v>
+        <v>78</v>
       </c>
       <c r="B11" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>20</v>
+        <v>131</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>134</v>
+        <v>79</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>136</v>
+        <v>80</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>138</v>
+        <v>81</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>139</v>
+        <v>82</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>140</v>
+        <v>83</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>135</v>
+        <v>84</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>122</v>
+        <v>133</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>30</v>
+        <v>148</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>31</v>
+        <v>144</v>
       </c>
       <c r="B22" t="s">
-        <v>32</v>
+        <v>135</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B23" t="s">
-        <v>34</v>
+        <v>115</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="B24" t="s">
-        <v>18</v>
+        <v>121</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="B25" t="s">
-        <v>37</v>
+        <v>149</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>38</v>
+        <v>24</v>
       </c>
       <c r="B26" t="s">
-        <v>39</v>
+        <v>85</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="B27" t="s">
-        <v>41</v>
+        <v>86</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>42</v>
+        <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>43</v>
+        <v>87</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>44</v>
+        <v>27</v>
       </c>
       <c r="B29" t="s">
-        <v>45</v>
+        <v>88</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>46</v>
+        <v>28</v>
       </c>
       <c r="B30" t="s">
-        <v>47</v>
+        <v>89</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>48</v>
+        <v>29</v>
       </c>
       <c r="B31" t="s">
-        <v>49</v>
+        <v>90</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>51</v>
+        <v>91</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>52</v>
+        <v>31</v>
       </c>
       <c r="B33" t="s">
-        <v>53</v>
+        <v>92</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>54</v>
+        <v>32</v>
       </c>
       <c r="B34" t="s">
-        <v>55</v>
+        <v>93</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>56</v>
+        <v>33</v>
       </c>
       <c r="B35" t="s">
-        <v>57</v>
+        <v>94</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>58</v>
+        <v>34</v>
       </c>
       <c r="B36" t="s">
-        <v>59</v>
+        <v>95</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>60</v>
+        <v>35</v>
       </c>
       <c r="B37" t="s">
-        <v>61</v>
+        <v>119</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>62</v>
+        <v>142</v>
       </c>
       <c r="B38" t="s">
-        <v>63</v>
+        <v>120</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>64</v>
+        <v>36</v>
       </c>
       <c r="B39" t="s">
-        <v>65</v>
+        <v>104</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>66</v>
+        <v>37</v>
       </c>
       <c r="B40" t="s">
-        <v>67</v>
+        <v>143</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>68</v>
+        <v>38</v>
       </c>
       <c r="B41" t="s">
-        <v>69</v>
+        <v>105</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>70</v>
+        <v>39</v>
       </c>
       <c r="B42" t="s">
-        <v>123</v>
+        <v>106</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>71</v>
+        <v>40</v>
       </c>
       <c r="B43" t="s">
-        <v>124</v>
+        <v>107</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>72</v>
+        <v>41</v>
       </c>
       <c r="B44" t="s">
-        <v>73</v>
+        <v>108</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>74</v>
+        <v>42</v>
       </c>
       <c r="B45" t="s">
-        <v>75</v>
+        <v>109</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>76</v>
+        <v>139</v>
       </c>
       <c r="B46" t="s">
-        <v>119</v>
+        <v>138</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>77</v>
+        <v>43</v>
       </c>
       <c r="B47" t="s">
-        <v>125</v>
+        <v>110</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>78</v>
+        <v>44</v>
       </c>
       <c r="B48" t="s">
-        <v>79</v>
+        <v>111</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>80</v>
+        <v>45</v>
       </c>
       <c r="B49" t="s">
-        <v>126</v>
+        <v>112</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>81</v>
+        <v>46</v>
       </c>
       <c r="B50" t="s">
-        <v>127</v>
+        <v>113</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>82</v>
+        <v>47</v>
       </c>
       <c r="B51" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>83</v>
+        <v>147</v>
       </c>
       <c r="B52" t="s">
-        <v>120</v>
+        <v>137</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>84</v>
+        <v>48</v>
       </c>
       <c r="B53" t="s">
-        <v>85</v>
+        <v>132</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>86</v>
+        <v>49</v>
       </c>
       <c r="B54" t="s">
-        <v>128</v>
+        <v>114</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>87</v>
+        <v>50</v>
       </c>
       <c r="B55" t="s">
-        <v>88</v>
+        <v>116</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>89</v>
+        <v>51</v>
       </c>
       <c r="B56" t="s">
-        <v>132</v>
+        <v>117</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>90</v>
+        <v>53</v>
       </c>
       <c r="B57" t="s">
-        <v>131</v>
+        <v>118</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>91</v>
+        <v>146</v>
       </c>
       <c r="B58" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A59" t="s">
-        <v>93</v>
-      </c>
-      <c r="B59" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A60" t="s">
-        <v>94</v>
-      </c>
-      <c r="B60" t="s">
-        <v>129</v>
+        <v>140</v>
       </c>
     </row>
   </sheetData>
@@ -1287,7 +1290,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:B76"/>
+  <dimension ref="A1:B77"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="42.77734375" customWidth="1"/>
@@ -1298,617 +1301,628 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>95</v>
+        <v>54</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>96</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>96</v>
+        <v>56</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>97</v>
+        <v>55</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>96</v>
+        <v>55</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>98</v>
+        <v>57</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>99</v>
+        <v>58</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>100</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>100</v>
+        <v>59</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="B10" t="s">
-        <v>101</v>
+        <v>60</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="B11" t="s">
-        <v>102</v>
+        <v>61</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="B12" t="s">
-        <v>97</v>
+        <v>56</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>17</v>
+        <v>52</v>
       </c>
       <c r="B13" t="s">
-        <v>102</v>
+        <v>60</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>141</v>
+        <v>11</v>
       </c>
       <c r="B14" t="s">
-        <v>103</v>
+        <v>62</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="B15" t="s">
-        <v>103</v>
+        <v>63</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>19</v>
+        <v>78</v>
       </c>
       <c r="B16" t="s">
-        <v>104</v>
+        <v>62</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="B17" t="s">
-        <v>105</v>
+        <v>64</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="B18" t="s">
-        <v>106</v>
+        <v>65</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="B19" t="s">
-        <v>106</v>
+        <v>65</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="B20" t="s">
-        <v>106</v>
+        <v>65</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="B21" t="s">
-        <v>105</v>
+        <v>64</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="B22" t="s">
-        <v>106</v>
+        <v>65</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="B23" t="s">
-        <v>106</v>
+        <v>65</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="B24" t="s">
-        <v>106</v>
+        <v>65</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="B25" t="s">
-        <v>106</v>
+        <v>65</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="B26" t="s">
-        <v>104</v>
+        <v>63</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="B27" t="s">
-        <v>101</v>
+        <v>60</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="B28" t="s">
-        <v>97</v>
+        <v>61</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="B29" t="s">
-        <v>98</v>
+        <v>59</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="B30" t="s">
-        <v>99</v>
+        <v>56</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>31</v>
+        <v>144</v>
       </c>
       <c r="B31" t="s">
-        <v>100</v>
+        <v>57</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>33</v>
+        <v>144</v>
       </c>
       <c r="B32" t="s">
-        <v>100</v>
+        <v>58</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>35</v>
+        <v>144</v>
       </c>
       <c r="B33" t="s">
-        <v>105</v>
+        <v>59</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>36</v>
+        <v>22</v>
       </c>
       <c r="B34" t="s">
-        <v>105</v>
+        <v>64</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="B35" t="s">
-        <v>105</v>
+        <v>64</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>40</v>
+        <v>24</v>
       </c>
       <c r="B36" t="s">
-        <v>105</v>
+        <v>64</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="B37" t="s">
-        <v>101</v>
+        <v>64</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>44</v>
+        <v>26</v>
       </c>
       <c r="B38" t="s">
-        <v>105</v>
+        <v>60</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>46</v>
+        <v>27</v>
       </c>
       <c r="B39" t="s">
-        <v>105</v>
+        <v>64</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>46</v>
+        <v>29</v>
       </c>
       <c r="B40" t="s">
-        <v>101</v>
+        <v>60</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>48</v>
+        <v>30</v>
       </c>
       <c r="B41" t="s">
-        <v>101</v>
+        <v>60</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>50</v>
+        <v>28</v>
       </c>
       <c r="B42" t="s">
-        <v>101</v>
+        <v>64</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="B43" t="s">
-        <v>105</v>
+        <v>60</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>54</v>
+        <v>31</v>
       </c>
       <c r="B44" t="s">
-        <v>105</v>
+        <v>64</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>56</v>
+        <v>32</v>
       </c>
       <c r="B45" t="s">
-        <v>101</v>
+        <v>64</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>58</v>
+        <v>33</v>
       </c>
       <c r="B46" t="s">
-        <v>105</v>
+        <v>60</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>60</v>
+        <v>34</v>
       </c>
       <c r="B47" t="s">
-        <v>102</v>
+        <v>64</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>62</v>
+        <v>53</v>
       </c>
       <c r="B48" t="s">
-        <v>101</v>
+        <v>60</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>64</v>
+        <v>142</v>
       </c>
       <c r="B49" t="s">
-        <v>101</v>
+        <v>60</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>66</v>
+        <v>36</v>
       </c>
       <c r="B50" t="s">
-        <v>98</v>
+        <v>60</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>66</v>
+        <v>37</v>
       </c>
       <c r="B51" t="s">
-        <v>99</v>
+        <v>57</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>66</v>
+        <v>37</v>
       </c>
       <c r="B52" t="s">
-        <v>103</v>
+        <v>58</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>68</v>
+        <v>37</v>
       </c>
       <c r="B53" t="s">
-        <v>98</v>
+        <v>62</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>68</v>
+        <v>35</v>
       </c>
       <c r="B54" t="s">
-        <v>99</v>
+        <v>61</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>68</v>
+        <v>146</v>
       </c>
       <c r="B55" t="s">
-        <v>100</v>
+        <v>59</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="B56" t="s">
-        <v>102</v>
+        <v>56</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>71</v>
+        <v>38</v>
       </c>
       <c r="B57" t="s">
-        <v>102</v>
+        <v>57</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>72</v>
+        <v>38</v>
       </c>
       <c r="B58" t="s">
-        <v>97</v>
+        <v>58</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>74</v>
+        <v>38</v>
       </c>
       <c r="B59" t="s">
-        <v>105</v>
+        <v>59</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>76</v>
+        <v>39</v>
       </c>
       <c r="B60" t="s">
-        <v>107</v>
+        <v>61</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>77</v>
+        <v>42</v>
       </c>
       <c r="B61" t="s">
-        <v>105</v>
+        <v>64</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>78</v>
+        <v>139</v>
       </c>
       <c r="B62" t="s">
-        <v>97</v>
+        <v>66</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="B63" t="s">
-        <v>97</v>
+        <v>61</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>80</v>
+        <v>43</v>
       </c>
       <c r="B64" t="s">
-        <v>96</v>
+        <v>64</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>81</v>
+        <v>44</v>
       </c>
       <c r="B65" t="s">
-        <v>97</v>
+        <v>56</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>81</v>
+        <v>45</v>
       </c>
       <c r="B66" t="s">
-        <v>96</v>
+        <v>56</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>82</v>
+        <v>45</v>
       </c>
       <c r="B67" t="s">
-        <v>105</v>
+        <v>55</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>83</v>
+        <v>47</v>
       </c>
       <c r="B68" t="s">
-        <v>105</v>
+        <v>59</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>84</v>
+        <v>47</v>
       </c>
       <c r="B69" t="s">
-        <v>100</v>
+        <v>64</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>86</v>
+        <v>46</v>
       </c>
       <c r="B70" t="s">
-        <v>101</v>
+        <v>56</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>87</v>
+        <v>46</v>
       </c>
       <c r="B71" t="s">
-        <v>101</v>
+        <v>55</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>89</v>
+        <v>147</v>
       </c>
       <c r="B72" t="s">
-        <v>96</v>
+        <v>64</v>
       </c>
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="B73" t="s">
-        <v>101</v>
+        <v>54</v>
       </c>
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
-        <v>91</v>
+        <v>48</v>
       </c>
       <c r="B74" t="s">
-        <v>101</v>
+        <v>59</v>
       </c>
     </row>
     <row r="75" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
-        <v>93</v>
+        <v>49</v>
       </c>
       <c r="B75" t="s">
-        <v>100</v>
+        <v>60</v>
       </c>
     </row>
     <row r="76" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
-        <v>94</v>
+        <v>50</v>
       </c>
       <c r="B76" t="s">
-        <v>100</v>
+        <v>60</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A77" t="s">
+        <v>51</v>
+      </c>
+      <c r="B77" t="s">
+        <v>55</v>
       </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B77">
+    <sortCondition ref="A2:A77"/>
+  </sortState>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:B60"/>
+  <dimension ref="A1:B59"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="32.5546875" customWidth="1"/>
@@ -1920,7 +1934,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>108</v>
+        <v>67</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
@@ -1928,7 +1942,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>109</v>
+        <v>68</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
@@ -1936,466 +1950,515 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>109</v>
+        <v>68</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>109</v>
+        <v>68</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>109</v>
+        <v>68</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>110</v>
+        <v>68</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B7" t="s">
-        <v>111</v>
+        <v>68</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B8" t="s">
-        <v>109</v>
+        <v>68</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="B9" t="s">
-        <v>109</v>
+        <v>68</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B10" t="s">
-        <v>109</v>
+        <v>68</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>141</v>
+        <v>22</v>
       </c>
       <c r="B11" t="s">
-        <v>112</v>
+        <v>68</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B12" t="s">
-        <v>112</v>
+        <v>68</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>21</v>
+        <v>35</v>
       </c>
       <c r="B13" t="s">
-        <v>109</v>
+        <v>68</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>22</v>
+        <v>41</v>
       </c>
       <c r="B14" t="s">
-        <v>110</v>
+        <v>68</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>23</v>
+        <v>39</v>
       </c>
       <c r="B15" t="s">
-        <v>113</v>
+        <v>68</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="B16" t="s">
-        <v>111</v>
+        <v>68</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>25</v>
+        <v>43</v>
       </c>
       <c r="B17" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="B18" t="s">
-        <v>112</v>
+        <v>68</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="B19" t="s">
-        <v>114</v>
+        <v>68</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="B20" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>29</v>
+        <v>6</v>
       </c>
       <c r="B21" t="s">
-        <v>109</v>
+        <v>69</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="B22" t="s">
-        <v>110</v>
+        <v>69</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>33</v>
+        <v>144</v>
       </c>
       <c r="B23" t="s">
-        <v>115</v>
+        <v>69</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>35</v>
+        <v>24</v>
       </c>
       <c r="B24" t="s">
-        <v>109</v>
+        <v>69</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B25" t="s">
-        <v>109</v>
+        <v>69</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="B26" t="s">
-        <v>110</v>
+        <v>69</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>40</v>
+        <v>21</v>
       </c>
       <c r="B27" t="s">
-        <v>115</v>
+        <v>74</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="B28" t="s">
-        <v>113</v>
+        <v>74</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>44</v>
+        <v>146</v>
       </c>
       <c r="B29" t="s">
-        <v>111</v>
+        <v>74</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>46</v>
+        <v>14</v>
       </c>
       <c r="B30" t="s">
-        <v>60</v>
+        <v>72</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>48</v>
+        <v>26</v>
       </c>
       <c r="B31" t="s">
-        <v>112</v>
+        <v>72</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="B32" t="s">
-        <v>116</v>
+        <v>72</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>52</v>
+        <v>7</v>
       </c>
       <c r="B33" t="s">
-        <v>117</v>
+        <v>70</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>54</v>
+        <v>15</v>
       </c>
       <c r="B34" t="s">
-        <v>84</v>
+        <v>70</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>56</v>
+        <v>27</v>
       </c>
       <c r="B35" t="s">
-        <v>114</v>
+        <v>70</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="B36" t="s">
-        <v>118</v>
+        <v>71</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>60</v>
+        <v>11</v>
       </c>
       <c r="B37" t="s">
-        <v>109</v>
+        <v>71</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="B38" t="s">
-        <v>112</v>
+        <v>71</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>64</v>
+        <v>17</v>
       </c>
       <c r="B39" t="s">
-        <v>112</v>
+        <v>71</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>66</v>
+        <v>29</v>
       </c>
       <c r="B40" t="s">
-        <v>113</v>
+        <v>71</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>68</v>
+        <v>142</v>
       </c>
       <c r="B41" t="s">
-        <v>110</v>
+        <v>71</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>70</v>
+        <v>36</v>
       </c>
       <c r="B42" t="s">
-        <v>109</v>
+        <v>71</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>71</v>
+        <v>30</v>
       </c>
       <c r="B43" t="s">
-        <v>109</v>
+        <v>75</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>72</v>
+        <v>53</v>
       </c>
       <c r="B44" t="s">
-        <v>109</v>
+        <v>75</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>74</v>
+        <v>16</v>
       </c>
       <c r="B45" t="s">
-        <v>60</v>
+        <v>35</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>76</v>
+        <v>19</v>
       </c>
       <c r="B46" t="s">
-        <v>117</v>
+        <v>35</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>77</v>
+        <v>28</v>
       </c>
       <c r="B47" t="s">
-        <v>109</v>
+        <v>35</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>78</v>
+        <v>42</v>
       </c>
       <c r="B48" t="s">
-        <v>109</v>
+        <v>35</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>80</v>
+        <v>31</v>
       </c>
       <c r="B49" t="s">
-        <v>109</v>
+        <v>76</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>81</v>
+        <v>139</v>
       </c>
       <c r="B50" t="s">
-        <v>109</v>
+        <v>76</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>82</v>
+        <v>147</v>
       </c>
       <c r="B51" t="s">
-        <v>110</v>
+        <v>76</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>83</v>
+        <v>32</v>
       </c>
       <c r="B52" t="s">
-        <v>117</v>
+        <v>48</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>84</v>
+        <v>48</v>
       </c>
       <c r="B53" t="s">
-        <v>84</v>
+        <v>48</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>86</v>
+        <v>18</v>
       </c>
       <c r="B54" t="s">
-        <v>114</v>
+        <v>73</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>87</v>
+        <v>33</v>
       </c>
       <c r="B55" t="s">
-        <v>118</v>
+        <v>73</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>89</v>
+        <v>49</v>
       </c>
       <c r="B56" t="s">
-        <v>118</v>
+        <v>73</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>90</v>
+        <v>34</v>
       </c>
       <c r="B57" t="s">
-        <v>112</v>
+        <v>77</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>91</v>
+        <v>50</v>
       </c>
       <c r="B58" t="s">
-        <v>116</v>
+        <v>77</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>93</v>
+        <v>51</v>
       </c>
       <c r="B59" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A60" t="s">
-        <v>94</v>
-      </c>
-      <c r="B60" t="s">
-        <v>110</v>
+        <v>77</v>
       </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:B59">
+    <sortCondition ref="B2:B59"/>
+  </sortState>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9D98AEF-5432-4436-ABD1-076D9C267FBE}">
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="19.109375" customWidth="1"/>
+    <col min="2" max="2" width="47.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>126</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B2" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>123</v>
+      </c>
+      <c r="B3" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>124</v>
+      </c>
+      <c r="B4" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>125</v>
+      </c>
+      <c r="B5" t="s">
+        <v>127</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>